<commit_message>
The tailed sign in the 1789 register, Haul. Lazy., and a spot sheet for the summons
Kalisz Tab.21: the stroke the editor first read as e-ogonek at the end of
four names is the clerk's sign for an ending such as -skiego (editor);
given as a colon like the same sign elsewhere: Kiedrow: (twice),
Trzebieslaw:, Siedlisk:. Text, English and clean workbook remade.

AGAD 1/169/0/1/1745, no. 150, "Haul. Lazy.": probably the Lazinskie
Oledry, not the village of Lazy (editor). Recorded, not matched.

APP 53/968/0/-/783: the spot sheet "Pen marks on the summons", six rows
with pictures (the margin name for no. 58, nos. 7, 53-55, 70, and the
note of costs); its rows copied to the holding's intake/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/units/app53640kalisztab21/APP_53_64_0_Kalisz_Tab_21_register.xlsx
+++ b/units/app53640kalisztab21/APP_53_64_0_Kalisz_Tab_21_register.xlsx
@@ -2413,7 +2413,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Dzierzawa Trzebiesławę</t>
+          <t>Dzierzawa Trzebiesław:</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>The last letter is written with a long tail; the editor reads it as ę.</t>
+          <t>The last word is shortened with the tailed sign that stands for an ending such as -skiego (editor, 2026-10-14); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Czachory Część Anto: Kiedrowę</t>
+          <t>Czachory Część Anto: Kiedrow:</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="H132" s="5" t="inlineStr">
         <is>
-          <t>The last letter is written with a long tail; the editor reads it as ę.</t>
+          <t>The last word is shortened with the tailed sign that stands for an ending such as -skiego (editor, 2026-10-14); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>z Części w Gołuchowie Kiedrowę</t>
+          <t>z Części w Gołuchowie Kiedrow:</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
-          <t>The last letter is written with a long tail; the editor reads it as ę.</t>
+          <t>The last word is shortened with the tailed sign that stands for an ending such as -skiego (editor, 2026-10-14); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Kuznica z Dąmbrową y Siedliskę</t>
+          <t>Kuznica z Dąmbrową y Siedlisk:</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="H231" s="5" t="inlineStr">
         <is>
-          <t>The last word is shortened with a flourish.</t>
+          <t>The last word is shortened with the tailed sign, here for the ending -iem (z Siedliskiem); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -10145,7 +10145,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Lease Trzebiesławę</t>
+          <t>Lease Trzebiesław:</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -10153,7 +10153,7 @@
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>The last letter is written with a long tail; the editor reads it as ę.</t>
+          <t>The last word is shortened with the tailed sign that stands for an ending such as -skiego (editor, 2026-10-14); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -10701,7 +10701,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Czachory part of Anto: Kiedrowę</t>
+          <t>Czachory part of Anto: Kiedrow:</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -10712,7 +10712,7 @@
       </c>
       <c r="H132" s="5" t="inlineStr">
         <is>
-          <t>The last letter is written with a long tail; the editor reads it as ę.</t>
+          <t>The last word is shortened with the tailed sign that stands for an ending such as -skiego (editor, 2026-10-14); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>From the part at Gołuchowie Kiedrowę</t>
+          <t>From the part at Gołuchowie Kiedrow:</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -10735,7 +10735,7 @@
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
-          <t>The last letter is written with a long tail; the editor reads it as ę.</t>
+          <t>The last word is shortened with the tailed sign that stands for an ending such as -skiego (editor, 2026-10-14); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>
@@ -12644,7 +12644,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Kuznica with Dąmbrową and Siedliskę</t>
+          <t>Kuznica with Dąmbrową and Siedlisk:</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -12655,7 +12655,7 @@
       </c>
       <c r="H231" s="5" t="inlineStr">
         <is>
-          <t>The last word is shortened with a flourish.</t>
+          <t>The last word is shortened with the tailed sign, here for the ending -iem (z Siedliskiem); given as a colon, as elsewhere in the register.</t>
         </is>
       </c>
     </row>

</xml_diff>